<commit_message>
Publish public research tools page
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Ra982ea540cb3437d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R73cdca6946c34539"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Rf6b755b686324be3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R4ce1fb746750422f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -44385,7 +44385,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaac97334d08475d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9836efac66e74a6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44554,7 +44554,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B22" s="27" t="str">
-        <x:v>e11a382425915e4242010d581867fade379cf7d2552bb3e1f475521ad5601c91</x:v>
+        <x:v>c38a1e075d9976ea234f0513844269a0bf320396912ad01f6e8cbe2436f3d689</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
@@ -44562,7 +44562,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>8f09eeed95250938a395b27c64b561a3dc4194208aac36e685902b281f13b0e2</x:v>
+        <x:v>c3e28863ef5ca2394dcc84c576ef3576b0e1bf44b193bf51d896a814713c86d4</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Clarify platform label differences
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R666c9ee77f52460f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R6709852dac51457f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R64e06212abf14915"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R007f0e7ca0a44da1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43827,7 +43827,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra493638b4a774839"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ffd77ab96574448"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43996,7 +43996,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B22" s="27" t="str">
-        <x:v>b9a25747acd45fda8b1d87350e7a56cf3062296d7bad0012f22b0a40395e8b4b</x:v>
+        <x:v>c61fb70214174cc554075ef38b2bcf49596000be1fb346abf819063621d58a6a</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
@@ -44004,7 +44004,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>7420b93fc431cba1af71cb213eeb4a55e0a809716b4de5383041cbd46c00e528</x:v>
+        <x:v>88d0673fc598f08275abc59d7b065cf84cc847217e977a788facfe4647c84b97</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Remove redundant Bangumi status filter
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R64e06212abf14915"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R007f0e7ca0a44da1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R593c80242dc444bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rf07e35ee77f34a35"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43827,7 +43827,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ffd77ab96574448"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cadcd9313894ea2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43996,7 +43996,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B22" s="27" t="str">
-        <x:v>c61fb70214174cc554075ef38b2bcf49596000be1fb346abf819063621d58a6a</x:v>
+        <x:v>0e53500e02bd980d75759b24c2b11b63628a0f12b3ff037228029424f1b439ca</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
@@ -44004,7 +44004,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>88d0673fc598f08275abc59d7b065cf84cc847217e977a788facfe4647c84b97</x:v>
+        <x:v>46676f3681a22fed60ceec4fd41b5312c03833848da523b8a1d402888c3178c0</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish relationship compression analysis
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R05fef613e1ef4fa7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R12f734399ceb4f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R79f1365e58a14abc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R752dd0d741c34525"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -521,26 +521,26 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="23.75" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="13.75" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13.130000114440918" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="15.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="15.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22.5" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="15.75" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="18.1299991607666" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="18.1299991607666" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="22.5" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="17.5" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="41.25" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="15" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="12.5" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="17.5" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="15" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="15.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="17.5" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="21.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="13.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="15.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="36.66999816894531" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="13.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="15.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="13.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="13.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="15.5600004196167" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
@@ -43827,7 +43827,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4855769915b4a3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18a502dceb6a479b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43836,9 +43836,9 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="25.6299991607666" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="71.25" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="2.25" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="63.33000183105469" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="2" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
@@ -43996,7 +43996,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B22" s="27" t="str">
-        <x:v>7bdc2bac3b137cecc8fa37079920e4face1376b3c91e127d2e83f8fbcaa6bcce</x:v>
+        <x:v>57898bc67e755ef933e29d1983bf8c2ba7e1e8ba7006bca1f7222b3f67772a8b</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
@@ -44004,7 +44004,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>601ef68883470fa5d2be9909342cd3e7b41636bf788737f5f7c319932ab8cd67</x:v>
+        <x:v>f9f28a5914c49a4d81559b65c8a0d8491be268fe38f584f969062ffa432a54bb</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Version public catalog requests
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R79f1365e58a14abc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R752dd0d741c34525"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R59155ccd91964930"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R235a6a0e8ec148a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43827,7 +43827,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18a502dceb6a479b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4678dd6b491945dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43996,7 +43996,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B22" s="27" t="str">
-        <x:v>57898bc67e755ef933e29d1983bf8c2ba7e1e8ba7006bca1f7222b3f67772a8b</x:v>
+        <x:v>972b5b8130c04de1b5cae923083e12c6acf2b7b4979f6bb5dfcc1d93c5376cdf</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
@@ -44004,7 +44004,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>f9f28a5914c49a4d81559b65c8a0d8491be268fe38f584f969062ffa432a54bb</x:v>
+        <x:v>3df899b45eca0812a5a6a29466bf81d1686b79c3959563a1f93e1122413fa3d5</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Make relationship filters orthogonal
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R59155ccd91964930"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R235a6a0e8ec148a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R9720a2b1d9fa441c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rbbfeea7ce98c4738"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43827,7 +43827,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4678dd6b491945dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4cf62fc5cc84343"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43996,7 +43996,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B22" s="27" t="str">
-        <x:v>972b5b8130c04de1b5cae923083e12c6acf2b7b4979f6bb5dfcc1d93c5376cdf</x:v>
+        <x:v>65c29e2f9c107cc19e560482f5d3448039da0fb2e49d0f26bcbe0fd074e2d384</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
@@ -44004,7 +44004,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>3df899b45eca0812a5a6a29466bf81d1686b79c3959563a1f93e1122413fa3d5</x:v>
+        <x:v>19a5fb0e6d491bb271a89dc4acf92d5a5121dc7894a4f6c9794ae9ede36e1b44</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Order relationship filter options
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R9720a2b1d9fa441c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rbbfeea7ce98c4738"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Ra74fd23afdd7495d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rca3c7832dfc0487e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43827,7 +43827,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4cf62fc5cc84343"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4b26f3677804f65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43996,7 +43996,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B22" s="27" t="str">
-        <x:v>65c29e2f9c107cc19e560482f5d3448039da0fb2e49d0f26bcbe0fd074e2d384</x:v>
+        <x:v>7cf502cd3ead8f15d3cc5ea9cf393d0c789a84a4db3f9e1549426134a7360ccc</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
@@ -44004,7 +44004,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>19a5fb0e6d491bb271a89dc4acf92d5a5121dc7894a4f6c9794ae9ede36e1b44</x:v>
+        <x:v>ea82041e3cbb38cd047f59c5ec34806edf5fe4e22dbd16e33d9eb86486246211</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Rename archive basis conclusion label
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Ra74fd23afdd7495d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rca3c7832dfc0487e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R073cf1183f1347ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R918a410d1c4743e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -303,7 +303,7 @@
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="作品名称"/>
     <x:tableColumn id="2" name="女女关系层级"/>
-    <x:tableColumn id="3" name="百合归档依据"/>
+    <x:tableColumn id="3" name="百合归档结论"/>
     <x:tableColumn id="4" name="女女恋爱位置"/>
     <x:tableColumn id="5" name="女女关系最高明确度"/>
     <x:tableColumn id="6" name="关系构成"/>
@@ -599,7 +599,7 @@
         <x:v>女女关系层级</x:v>
       </x:c>
       <x:c r="C4" s="44" t="str">
-        <x:v>百合归档依据</x:v>
+        <x:v>百合归档结论</x:v>
       </x:c>
       <x:c r="D4" s="44" t="str">
         <x:v>女女恋爱位置</x:v>
@@ -43827,7 +43827,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4b26f3677804f65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra204c32af4de4281"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43913,7 +43913,7 @@
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
       <x:c r="A11" s="27" t="str">
-        <x:v>百合归档依据</x:v>
+        <x:v>百合归档结论</x:v>
       </x:c>
       <x:c r="B11" s="27" t="str">
         <x:v>说明是作品分类、读者解读、非百合或证据不足，不能由单一标签替代。</x:v>
@@ -43996,7 +43996,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B22" s="27" t="str">
-        <x:v>7cf502cd3ead8f15d3cc5ea9cf393d0c789a84a4db3f9e1549426134a7360ccc</x:v>
+        <x:v>f188437be8a903101ca9608319d2d2e944c6bb960011b394522f8279748cc609</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
@@ -44004,7 +44004,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>ea82041e3cbb38cd047f59c5ec34806edf5fe4e22dbd16e33d9eb86486246211</x:v>
+        <x:v>7bfa0cc694aca983e834e5b56aa89f1421fcca69faf46c44e1295a5e3884c964</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Add main explicit desire query
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Rd00aef9dd3bb4a4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R912b47fa08e3469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R3acbc759a24742f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R2ee6f9eaff82427b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45921,7 +45921,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf86fa24f41a489c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4feac85674754d19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46098,7 +46098,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>2ea9c897fa11d64f31ca0b750efad695f53e0eabdc6d6308813e7923a7cd9b9c</x:v>
+        <x:v>dcdbb92b1fba02bf8489dab84ce8a7a9019779c2358478ef10a1a47b200cd690</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -46106,7 +46106,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>2b8c2b02ea268a71a9e93d592f203662f4c780e27af606ef76d8eaf09755840d</x:v>
+        <x:v>8b5872a64dd145218308669186927671d971756467dd36e9de0b3398bede036d</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Improve catalog filters and workbook access
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R3acbc759a24742f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R2ee6f9eaff82427b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R2af57f1edad0468e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R0fa1229a00a841c8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -571,7 +571,7 @@
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>数据快照日期为 2026-08-10。分类字段来自正篇材料的分层判断；官方证据与四个数据库字段用于对照，不是对作品关系的投票或裁决。</x:v>
+        <x:v>数据快照日期为 2026-08-11。分类字段来自正篇材料的分层判断；官方证据与四个数据库字段用于对照，不是对作品关系的投票或裁决。</x:v>
       </x:c>
       <x:c r="B2" s="9"/>
       <x:c r="C2" s="9"/>
@@ -45921,7 +45921,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4feac85674754d19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dafc09db3584db4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45944,7 +45944,7 @@
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>比较快照日期：2026-08-10。AniList 相关度 0、无精确条目、未知、所核未见和资料不足不是同一个状态。</x:v>
+        <x:v>比较快照日期：2026-08-11。AniList 相关度 0、无精确条目、未知、所核未见和资料不足不是同一个状态。</x:v>
       </x:c>
       <x:c r="B2" s="9"/>
       <x:c r="C2" s="9"/>
@@ -46090,7 +46090,7 @@
         <x:v>数据日期</x:v>
       </x:c>
       <x:c r="B22" s="27" t="str">
-        <x:v>2026-08-10</x:v>
+        <x:v>2026-08-11</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
@@ -46098,7 +46098,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>dcdbb92b1fba02bf8489dab84ce8a7a9019779c2358478ef10a1a47b200cd690</x:v>
+        <x:v>d0e664d216eb817ec7a21a003947c631cb6e1b7791077ad2aa06a368a84f1515</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -46106,7 +46106,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>8b5872a64dd145218308669186927671d971756467dd36e9de0b3398bede036d</x:v>
+        <x:v>47c00884b207e9662ba5f978d6e72cbee93b0791bffe04cc9e5e3ddfe8ba75bd</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish localized report summaries
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R2af57f1edad0468e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R0fa1229a00a841c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R9b51337959cb4d9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rdbac9d420c4a4259"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45921,7 +45921,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dafc09db3584db4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9708b8f0e8f54ccf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46098,7 +46098,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>d0e664d216eb817ec7a21a003947c631cb6e1b7791077ad2aa06a368a84f1515</x:v>
+        <x:v>eb752e9258df91db4dd8f1897526361e6cd1c51da1a5566b806a9ec221646cee</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -46106,7 +46106,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>47c00884b207e9662ba5f978d6e72cbee93b0791bffe04cc9e5e3ddfe8ba75bd</x:v>
+        <x:v>da67c356d42fa4950cdd4d0271d71deae67a887c9ab79805195b5bf4e93bd334</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish relationship query reflection
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R9b51337959cb4d9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rdbac9d420c4a4259"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R9494c1d1e3d54966"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R1db8ad235a2a4688"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45921,7 +45921,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9708b8f0e8f54ccf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fa421bfe5cb4beb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46098,7 +46098,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>eb752e9258df91db4dd8f1897526361e6cd1c51da1a5566b806a9ec221646cee</x:v>
+        <x:v>d31292b3e9a8a2ea054db5b07bb4d1bb46cea30ced4b5fd9f3fbe13b7308c98c</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -46106,7 +46106,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>da67c356d42fa4950cdd4d0271d71deae67a887c9ab79805195b5bf4e93bd334</x:v>
+        <x:v>832cb39aa377feb02414730ca091cffd27927f297361a2e0e0f8fce63b48ee56</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish yuri concentration semantic audit
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R9494c1d1e3d54966"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R1db8ad235a2a4688"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R9df4f9ef98a64e34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rd00ab29cfc3c4d1b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45921,7 +45921,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fa421bfe5cb4beb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R551be0d654ae4aa6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46098,7 +46098,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>d31292b3e9a8a2ea054db5b07bb4d1bb46cea30ced4b5fd9f3fbe13b7308c98c</x:v>
+        <x:v>9ba8675897a2401370f5e78e043d6bc3e37260d3a78eccfca6a04b55739c511e</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -46106,7 +46106,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>832cb39aa377feb02414730ca091cffd27927f297361a2e0e0f8fce63b48ee56</x:v>
+        <x:v>b717d80d044766c070b4941dfd0007edb8f2edd6a887ae18434df2bc1434f075</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish relationship-aware archive queries
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R9df4f9ef98a64e34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rd00ab29cfc3c4d1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Re20b3daa5b964603"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R243d802ef6234ab7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -571,7 +571,7 @@
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>数据快照日期为 2026-08-11。分类字段来自正篇材料的分层判断；官方证据与四个数据库字段用于对照，不是对作品关系的投票或裁决。</x:v>
+        <x:v>数据快照日期为 2026-08-12。分类字段来自正篇材料的分层判断；官方证据与四个数据库字段用于对照，不是对作品关系的投票或裁决。</x:v>
       </x:c>
       <x:c r="B2" s="9"/>
       <x:c r="C2" s="9"/>
@@ -45921,7 +45921,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R551be0d654ae4aa6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R605e4f99913f41c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45944,7 +45944,7 @@
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>比较快照日期：2026-08-11。AniList 相关度 0、无精确条目、未知、所核未见和资料不足不是同一个状态。</x:v>
+        <x:v>比较快照日期：2026-08-12。AniList 相关度 0、无精确条目、未知、所核未见和资料不足不是同一个状态。</x:v>
       </x:c>
       <x:c r="B2" s="9"/>
       <x:c r="C2" s="9"/>
@@ -46090,7 +46090,7 @@
         <x:v>数据日期</x:v>
       </x:c>
       <x:c r="B22" s="27" t="str">
-        <x:v>2026-08-11</x:v>
+        <x:v>2026-08-12</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
@@ -46098,7 +46098,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>9ba8675897a2401370f5e78e043d6bc3e37260d3a78eccfca6a04b55739c511e</x:v>
+        <x:v>25b5f9cf5486cd4c978379417ed10e13fe4276f551482cb69809f366829ed52e</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -46106,7 +46106,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>b717d80d044766c070b4941dfd0007edb8f2edd6a887ae18434df2bc1434f075</x:v>
+        <x:v>93025a2e4c83213bb0aeee4f23ccf3c0eff6e8ce31df56233da543cce24fd5a3</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish non-romantic mainline query
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Re20b3daa5b964603"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R243d802ef6234ab7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R2c4a02816a004118"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R4716cfa15f9b44fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45921,7 +45921,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R605e4f99913f41c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8166577a253b46a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46098,7 +46098,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>25b5f9cf5486cd4c978379417ed10e13fe4276f551482cb69809f366829ed52e</x:v>
+        <x:v>2b0bd0c8a4f78f4b5704320be8d6432ad377331a14340c3362cba9973c6977f2</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -46106,7 +46106,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>93025a2e4c83213bb0aeee4f23ccf3c0eff6e8ce31df56233da543cce24fd5a3</x:v>
+        <x:v>46d9ec056d3473cb6c5e3cffad5156995d77351645ee45ef4bd8657dabdcbc9e</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish refreshed Anime-Planet coverage
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R2c4a02816a004118"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R4716cfa15f9b44fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R6148f65dd9d34fdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R55987b8174654be5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2860,7 +2860,7 @@
         <x:v>无</x:v>
       </x:c>
       <x:c r="S38" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T38" s="33" t="n">
         <x:v>0</x:v>
@@ -3250,7 +3250,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S44" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T44" s="33" t="str">
         <x:v>无精确条目</x:v>
@@ -4745,7 +4745,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S67" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T67" s="33" t="n">
         <x:v>0</x:v>
@@ -6630,7 +6630,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S96" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T96" s="33" t="n">
         <x:v>0</x:v>
@@ -7800,7 +7800,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S114" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>有</x:v>
       </x:c>
       <x:c r="T114" s="33" t="n">
         <x:v>82</x:v>
@@ -8450,7 +8450,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S124" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>有</x:v>
       </x:c>
       <x:c r="T124" s="33" t="n">
         <x:v>92</x:v>
@@ -10400,7 +10400,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S154" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T154" s="33" t="n">
         <x:v>0</x:v>
@@ -12935,7 +12935,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S193" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T193" s="33" t="n">
         <x:v>0</x:v>
@@ -15730,7 +15730,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S236" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T236" s="33" t="n">
         <x:v>0</x:v>
@@ -15795,7 +15795,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S237" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T237" s="33" t="n">
         <x:v>0</x:v>
@@ -16965,7 +16965,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S255" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T255" s="33" t="n">
         <x:v>60</x:v>
@@ -17225,7 +17225,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S259" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T259" s="33" t="n">
         <x:v>0</x:v>
@@ -17290,7 +17290,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S260" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T260" s="33" t="n">
         <x:v>0</x:v>
@@ -18915,7 +18915,7 @@
         <x:v>无</x:v>
       </x:c>
       <x:c r="S285" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T285" s="33" t="n">
         <x:v>0</x:v>
@@ -19175,7 +19175,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S289" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T289" s="33" t="n">
         <x:v>0</x:v>
@@ -20800,7 +20800,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S314" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>有</x:v>
       </x:c>
       <x:c r="T314" s="33" t="n">
         <x:v>60</x:v>
@@ -21840,7 +21840,7 @@
         <x:v>无</x:v>
       </x:c>
       <x:c r="S330" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T330" s="33" t="n">
         <x:v>0</x:v>
@@ -24895,7 +24895,7 @@
         <x:v>无</x:v>
       </x:c>
       <x:c r="S377" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T377" s="33" t="n">
         <x:v>73</x:v>
@@ -26000,7 +26000,7 @@
         <x:v>无</x:v>
       </x:c>
       <x:c r="S394" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T394" s="33" t="n">
         <x:v>79</x:v>
@@ -28665,7 +28665,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S435" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T435" s="33" t="n">
         <x:v>0</x:v>
@@ -31200,7 +31200,7 @@
         <x:v>无</x:v>
       </x:c>
       <x:c r="S474" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T474" s="33" t="n">
         <x:v>0</x:v>
@@ -31460,7 +31460,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S478" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T478" s="33" t="n">
         <x:v>0</x:v>
@@ -34385,7 +34385,7 @@
         <x:v>无</x:v>
       </x:c>
       <x:c r="S523" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T523" s="33" t="n">
         <x:v>0</x:v>
@@ -41730,7 +41730,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S636" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T636" s="33" t="n">
         <x:v>0</x:v>
@@ -42900,7 +42900,7 @@
         <x:v>无</x:v>
       </x:c>
       <x:c r="S654" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T654" s="33" t="n">
         <x:v>0</x:v>
@@ -43550,7 +43550,7 @@
         <x:v>无</x:v>
       </x:c>
       <x:c r="S664" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T664" s="33" t="n">
         <x:v>0</x:v>
@@ -44395,7 +44395,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S677" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T677" s="33" t="n">
         <x:v>80</x:v>
@@ -44785,7 +44785,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S683" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T683" s="33" t="n">
         <x:v>0</x:v>
@@ -45175,7 +45175,7 @@
         <x:v>无</x:v>
       </x:c>
       <x:c r="S689" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T689" s="33" t="n">
         <x:v>0</x:v>
@@ -45565,7 +45565,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S695" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T695" s="33" t="n">
         <x:v>50</x:v>
@@ -45890,7 +45890,7 @@
         <x:v>有</x:v>
       </x:c>
       <x:c r="S700" s="42" t="str">
-        <x:v>无精确条目</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="T700" s="33" t="n">
         <x:v>82</x:v>
@@ -45921,7 +45921,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8166577a253b46a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R750879fa290141e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46098,7 +46098,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>2b0bd0c8a4f78f4b5704320be8d6432ad377331a14340c3362cba9973c6977f2</x:v>
+        <x:v>d9fc4ccda1257f4bcd4143b0de86781839d24434325ccaaff65c809577b7bd5f</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -46106,7 +46106,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>46d9ec056d3473cb6c5e3cffad5156995d77351645ee45ef4bd8657dabdcbc9e</x:v>
+        <x:v>16b1a58ff8c886e9462ebff7104c9ee4aa50a850ad71158a483b15accc8fc1ed</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Add Bangumi tag filters
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R98bb68a2101c442a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R53e6f140ea0c4631"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R82f2c4b891414229"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R3eb16de2ef904ad0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45921,7 +45921,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad645e33efb1448b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd561dd96ebd4c36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46098,7 +46098,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>5541e693dbff228af9c51069dc01da70f0dfea6083df5daa7ad5a03c614a33e1</x:v>
+        <x:v>b2597285288a4135fed63ac782a4d8c72fb8be914a5b9976f07109b0c316bfbf</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -46106,7 +46106,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>bfdb9abdcc705ba10eef95279772dce93ecf1e11620852cbc450ea663d7bf95b</x:v>
+        <x:v>ffad010d783a393a71b04b10eb090bdbb9428c12c2b6f9f550be76c949fa2051</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Order public tags by work coverage
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R82f2c4b891414229"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R3eb16de2ef904ad0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R21041f07896b49c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rf880c5c049884079"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45921,7 +45921,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd561dd96ebd4c36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc77b1a9e2f24c8c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46098,7 +46098,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>b2597285288a4135fed63ac782a4d8c72fb8be914a5b9976f07109b0c316bfbf</x:v>
+        <x:v>624fc487457dc97d595020ca8baf11cc4946905639f4b58d60291d5704e74522</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -46106,7 +46106,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>ffad010d783a393a71b04b10eb090bdbb9428c12c2b6f9f550be76c949fa2051</x:v>
+        <x:v>79347de9f2fa1010b922cbf769a4aafa9a3093366fd57b4863c7e99b6df67a66</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish platform label comparison lookup
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R21041f07896b49c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rf880c5c049884079"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R7f55403cb4b64354"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R496d47cc438c46c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45921,7 +45921,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc77b1a9e2f24c8c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R413607d7477c4d74"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46098,7 +46098,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>624fc487457dc97d595020ca8baf11cc4946905639f4b58d60291d5704e74522</x:v>
+        <x:v>3033681825530d8ebf7992b045e8a1ae931af62507368f969212924d946ee7e1</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -46106,7 +46106,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>79347de9f2fa1010b922cbf769a4aafa9a3093366fd57b4863c7e99b6df67a66</x:v>
+        <x:v>58ff6be2317fc4d4702586953c68853382f3d5ee274268d2ffe7f500893d7e3e</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish expanded unified tag filters
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R0854c14ea8d3419f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R854dae80d2a3469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Re248ab33ecde4b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rfb5f86fe08d642ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45921,7 +45921,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58b0416c6f35448c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R379c3b35998948b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46098,7 +46098,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>22fbd76d76362a899adef377ec688d28528e2cd2009cbe9a8141ba6696c4df77</x:v>
+        <x:v>ee935d64d4781fa76daa5726df16c5a859ef5c92b8f85d4f7866ced168447305</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -46106,7 +46106,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>21bc9af39bbfc4f362ff9be15fc1472f560677535fec1c716f1b48bf1f9a6f65</x:v>
+        <x:v>6296482f51f505312122a33e33308600e6030fe596adf32a7aa4cf329e977cc6</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish work-page platform tags
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Re248ab33ecde4b45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rfb5f86fe08d642ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R8faea4aae7d94d42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R9768e08d45144631"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -571,7 +571,7 @@
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>数据快照日期为 2026-08-14。分类字段来自正篇材料的分层判断；官方证据与四个数据库字段用于对照，不是对作品关系的投票或裁决。</x:v>
+        <x:v>数据快照日期为 2026-08-15。分类字段来自正篇材料的分层判断；官方证据与四个数据库字段用于对照，不是对作品关系的投票或裁决。</x:v>
       </x:c>
       <x:c r="B2" s="9"/>
       <x:c r="C2" s="9"/>
@@ -26786,7 +26786,7 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="U406" s="27" t="str">
-        <x:v>无</x:v>
+        <x:v>无可对应条目</x:v>
       </x:c>
     </x:row>
     <x:row r="407" ht="57" customHeight="1">
@@ -45921,7 +45921,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R379c3b35998948b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R894f93594ee24e91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45944,7 +45944,7 @@
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>比较快照日期：2026-08-14。AniList 相关度 0、无可对应条目、未知、所核未见和资料不足不是同一个状态。</x:v>
+        <x:v>比较快照日期：2026-08-15。AniList 相关度 0、无可对应条目、未知、所核未见和资料不足不是同一个状态。</x:v>
       </x:c>
       <x:c r="B2" s="9"/>
       <x:c r="C2" s="9"/>
@@ -46090,7 +46090,7 @@
         <x:v>数据日期</x:v>
       </x:c>
       <x:c r="B22" s="27" t="str">
-        <x:v>2026-08-14</x:v>
+        <x:v>2026-08-15</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
@@ -46098,7 +46098,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>ee935d64d4781fa76daa5726df16c5a859ef5c92b8f85d4f7866ced168447305</x:v>
+        <x:v>37b32d6787ff0f29b77d61d7127aaaf2c4efa2eb4729c9235a72e8b282ba44d3</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -46106,7 +46106,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>6296482f51f505312122a33e33308600e6030fe596adf32a7aa4cf329e977cc6</x:v>
+        <x:v>3d548821be3dc7b77b38cd38d6b31d46322845a8cd7dbdd9fe9f13fc1e58687b</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Refresh platform vocabulary provenance
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R6aa3696808154c75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rdd4a5f08c8474041"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Ra6095689f3264a02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rb566acd3606845ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -52966,7 +52966,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a509f0fee0f458d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc77a69a78c645e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53143,7 +53143,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>2cdbb6dc0c843afc361d1b7f617dacf09376ecf89708b0bab8596070e4120ee9</x:v>
+        <x:v>3091d2e16e5c3be3fa6e64d783c6665bbfd32c9b1d2d873057283784c83dffb1</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -53151,7 +53151,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>316521cb180cf618e1698ab14ae99cef86013b38c9d425e867daccfb2d7dd0b4</x:v>
+        <x:v>45749d542bf282a6f6cb4a08102b50d763281da29a38d8b98dee80aff32c4546</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish default catalog filter and raw tag highlights
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Ra6095689f3264a02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rb566acd3606845ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R0fe6ccff246049be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Ra696d76ab7644fe9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -52966,7 +52966,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc77a69a78c645e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1258d4d5331542e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53143,7 +53143,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>3091d2e16e5c3be3fa6e64d783c6665bbfd32c9b1d2d873057283784c83dffb1</x:v>
+        <x:v>c6fd4080e6927c4865bb80dc214aa9708a1ea408b94240041d069dd49fb1004d</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -53151,7 +53151,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>45749d542bf282a6f6cb4a08102b50d763281da29a38d8b98dee80aff32c4546</x:v>
+        <x:v>12a3a28275ec583fddffa7b9f919d39539b570d340b7bf9b27f37bbabd9e92ae</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish Ikoku Nikki relationship revision
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R0fe6ccff246049be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Ra696d76ab7644fe9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Rb94dc656cdef4881"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R5f6e8e54779141f4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1317,19 +1317,19 @@
         <x:v>主线</x:v>
       </x:c>
       <x:c r="C15" s="30" t="str">
-        <x:v>非百合</x:v>
+        <x:v>文类外百合阅读</x:v>
       </x:c>
       <x:c r="D15" s="30" t="str">
-        <x:v>缺席</x:v>
+        <x:v>局部</x:v>
       </x:c>
       <x:c r="E15" s="30" t="str">
-        <x:v>非恋爱</x:v>
+        <x:v>潜在恋爱</x:v>
       </x:c>
       <x:c r="F15" s="30" t="str">
         <x:v>多组异质关系</x:v>
       </x:c>
       <x:c r="G15" s="30" t="str">
-        <x:v>范围内没有性取向身份依据</x:v>
+        <x:v>只有关系性质推断，无身份自述</x:v>
       </x:c>
       <x:c r="H15" s="30" t="str">
         <x:v>所核未见</x:v>
@@ -52966,7 +52966,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1258d4d5331542e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7311bb17d8e44d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53143,7 +53143,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>c6fd4080e6927c4865bb80dc214aa9708a1ea408b94240041d069dd49fb1004d</x:v>
+        <x:v>a53cd5cdeab249536db0c9fee420feea5ff531407e0c71654867565c1ab4c394</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -53151,7 +53151,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>12a3a28275ec583fddffa7b9f919d39539b570d340b7bf9b27f37bbabd9e92ae</x:v>
+        <x:v>f834fb02cb25d34c41bc800c93faac34afa3f01c8cb67aeac3907d741c7d3e5b</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish relation-aware snapshot filters
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Rb94dc656cdef4881"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R5f6e8e54779141f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Rf19496a45c084704"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R709552ad31f143df"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -52966,7 +52966,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7311bb17d8e44d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e38a5b5d4884db8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53143,7 +53143,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>a53cd5cdeab249536db0c9fee420feea5ff531407e0c71654867565c1ab4c394</x:v>
+        <x:v>df096331c35b5c8738723d45969c78150043ea90a76cbbc62a6e9c56e03867e4</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -53151,7 +53151,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>f834fb02cb25d34c41bc800c93faac34afa3f01c8cb67aeac3907d741c7d3e5b</x:v>
+        <x:v>65355fd12997a670e2f48daef0bc667d76cd3e20fe16cbdda9a5b54e90aa4656</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish revised platform analysis topics
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Rf19496a45c084704"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R709552ad31f143df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Rc28eeef9e7e247c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R9274e64f2207462d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -571,7 +571,7 @@
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>数据快照日期为 2026-08-16。分类字段来自正篇材料的分层判断；官方证据与四个数据库字段用于对照，不是对作品关系的投票或裁决。</x:v>
+        <x:v>数据快照日期为 2026-08-17。分类字段来自正篇材料的分层判断；官方证据与四个数据库字段用于对照，不是对作品关系的投票或裁决。</x:v>
       </x:c>
       <x:c r="B2" s="9"/>
       <x:c r="C2" s="9"/>
@@ -5120,7 +5120,7 @@
         <x:v>无</x:v>
       </x:c>
       <x:c r="N73" s="27" t="str">
-        <x:v>中学生角色的亲吻、婚姻和恋爱想象被用于喜剧，部分肢体接触与恋爱台词属于角色扮演或幻想。</x:v>
+        <x:v>中学生角色的亲吻、婚姻和恋爱想象被用于喜剧；姐妹之间的单向恋爱欲望及对衣物、洗澡和同床的迷恋也被用于喜剧。</x:v>
       </x:c>
       <x:c r="O73" s="30" t="str">
         <x:v>有可对应条目</x:v>
@@ -8668,13 +8668,13 @@
         <x:v>重要副线</x:v>
       </x:c>
       <x:c r="E128" s="30" t="str">
-        <x:v>潜在恋爱</x:v>
+        <x:v>明确女女恋爱欲望</x:v>
       </x:c>
       <x:c r="F128" s="30" t="str">
         <x:v>多组异质关系</x:v>
       </x:c>
       <x:c r="G128" s="30" t="str">
-        <x:v>只有关系性质推断，无身份自述</x:v>
+        <x:v>只有明确关系／欲望事实，无身份自述</x:v>
       </x:c>
       <x:c r="H128" s="30" t="str">
         <x:v>是</x:v>
@@ -9708,13 +9708,13 @@
         <x:v>重要副线</x:v>
       </x:c>
       <x:c r="E144" s="30" t="str">
-        <x:v>潜在恋爱</x:v>
+        <x:v>明确女女恋爱欲望</x:v>
       </x:c>
       <x:c r="F144" s="30" t="str">
         <x:v>多组异质关系</x:v>
       </x:c>
       <x:c r="G144" s="30" t="str">
-        <x:v>只有关系性质推断，无身份自述</x:v>
+        <x:v>只有明确关系／欲望事实，无身份自述</x:v>
       </x:c>
       <x:c r="H144" s="30" t="str">
         <x:v>是</x:v>
@@ -29010,7 +29010,7 @@
         <x:v>文类内百合</x:v>
       </x:c>
       <x:c r="D441" s="30" t="str">
-        <x:v>重要副线</x:v>
+        <x:v>局部</x:v>
       </x:c>
       <x:c r="E441" s="30" t="str">
         <x:v>明确女女恋爱欲望</x:v>
@@ -37590,7 +37590,7 @@
         <x:v>文类内百合</x:v>
       </x:c>
       <x:c r="D573" s="30" t="str">
-        <x:v>重要副线</x:v>
+        <x:v>主线</x:v>
       </x:c>
       <x:c r="E573" s="30" t="str">
         <x:v>明确女女交往关系</x:v>
@@ -46170,7 +46170,7 @@
         <x:v>文类内百合</x:v>
       </x:c>
       <x:c r="D705" s="30" t="str">
-        <x:v>重要副线</x:v>
+        <x:v>主线</x:v>
       </x:c>
       <x:c r="E705" s="30" t="str">
         <x:v>潜在恋爱</x:v>
@@ -52966,7 +52966,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e38a5b5d4884db8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R031a7025b6b3475c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -52989,7 +52989,7 @@
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>比较快照日期：2026-08-16。AniList 相关度 0、无可对应条目、未知、所核未见和资料不足不是同一个状态。</x:v>
+        <x:v>比较快照日期：2026-08-17。AniList 相关度 0、无可对应条目、未知、所核未见和资料不足不是同一个状态。</x:v>
       </x:c>
       <x:c r="B2" s="9"/>
       <x:c r="C2" s="9"/>
@@ -53135,7 +53135,7 @@
         <x:v>数据日期</x:v>
       </x:c>
       <x:c r="B22" s="27" t="str">
-        <x:v>2026-08-16</x:v>
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
@@ -53143,7 +53143,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>df096331c35b5c8738723d45969c78150043ea90a76cbbc62a6e9c56e03867e4</x:v>
+        <x:v>13d123675e692c2ce4699de7d74e4f78512b989cffcb7ecae8ec91f714bce3b7</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -53151,7 +53151,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>65355fd12997a670e2f48daef0bc667d76cd3e20fe16cbdda9a5b54e90aa4656</x:v>
+        <x:v>6e992e8bc8d9830f40af5561f3d1149f3b28861cba28b21f3650ee3a10ec927f</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Migrate release authority to schema 2
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Rc28eeef9e7e247c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R9274e64f2207462d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Ra32e87dcafd04c18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R5f88c871b5f14863"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -52966,7 +52966,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R031a7025b6b3475c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc128ec184384f6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53143,7 +53143,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>13d123675e692c2ce4699de7d74e4f78512b989cffcb7ecae8ec91f714bce3b7</x:v>
+        <x:v>6e1ec9771cb2f65af980168fd625824af115296ffd45c58982b4fc921bf4b180</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -53151,7 +53151,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>6e992e8bc8d9830f40af5561f3d1149f3b28861cba28b21f3650ee3a10ec927f</x:v>
+        <x:v>816c310a45d7fab72f6f63e7416f7e568d31444047fc1cf343552d712efeea65</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Publish platform label explicitness analysis
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="Ra32e87dcafd04c18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R5f88c871b5f14863"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R1624c2f30eda455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rfba004b48f7848fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -571,7 +571,7 @@
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>数据快照日期为 2026-08-17。分类字段来自正篇材料的分层判断；官方证据与四个数据库字段用于对照，不是对作品关系的投票或裁决。</x:v>
+        <x:v>数据快照日期为 2026-08-18。分类字段来自正篇材料的分层判断；官方证据与四个数据库字段用于对照，不是对作品关系的投票或裁决。</x:v>
       </x:c>
       <x:c r="B2" s="9"/>
       <x:c r="C2" s="9"/>
@@ -52966,7 +52966,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc128ec184384f6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc364b2d87a5846d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -52989,7 +52989,7 @@
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>比较快照日期：2026-08-17。AniList 相关度 0、无可对应条目、未知、所核未见和资料不足不是同一个状态。</x:v>
+        <x:v>比较快照日期：2026-08-18。AniList 相关度 0、无可对应条目、未知、所核未见和资料不足不是同一个状态。</x:v>
       </x:c>
       <x:c r="B2" s="9"/>
       <x:c r="C2" s="9"/>
@@ -53135,7 +53135,7 @@
         <x:v>数据日期</x:v>
       </x:c>
       <x:c r="B22" s="27" t="str">
-        <x:v>2026-08-17</x:v>
+        <x:v>2026-08-18</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
@@ -53143,7 +53143,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>6e1ec9771cb2f65af980168fd625824af115296ffd45c58982b4fc921bf4b180</x:v>
+        <x:v>6d4d1e1892417249d5ab6a1cb821b2390793ecdee9f7867e9f39bc2a97ff79d0</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -53151,7 +53151,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>816c310a45d7fab72f6f63e7416f7e568d31444047fc1cf343552d712efeea65</x:v>
+        <x:v>ee301e9668a48755b18b19cc7d5f57f711e73a1c1c5473f6828131b2320cd68b</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>